<commit_message>
nameroll1 update to 443
</commit_message>
<xml_diff>
--- a/test-site/nameroll1.xlsx
+++ b/test-site/nameroll1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\web-projects\test-site\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\web-projects\test-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D5CADA7-2F13-4444-87CC-7ABFB5D92472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4D8620E-941B-4A85-B1D2-0DFB2291139A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{23396267-709B-4E41-9020-7C481B582814}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="443">
   <si>
     <t>曹正烜</t>
   </si>
@@ -413,9 +413,6 @@
     <t>乙增婷</t>
   </si>
   <si>
-    <t>卲麗民</t>
-  </si>
-  <si>
     <t>莊建美</t>
   </si>
   <si>
@@ -440,9 +437,6 @@
     <t>陳瑞英</t>
   </si>
   <si>
-    <t>凃鳳英</t>
-  </si>
-  <si>
     <t>李英華</t>
   </si>
   <si>
@@ -704,12 +698,6 @@
     <t>周    萍</t>
   </si>
   <si>
-    <t>陳錦清</t>
-  </si>
-  <si>
-    <t>亞    蒂</t>
-  </si>
-  <si>
     <t>施純謚</t>
   </si>
   <si>
@@ -833,9 +821,6 @@
     <t>歐羅娜</t>
   </si>
   <si>
-    <t>李聖文</t>
-  </si>
-  <si>
     <t>李昀庭</t>
   </si>
   <si>
@@ -914,9 +899,6 @@
     <t>葉興漢</t>
   </si>
   <si>
-    <t>萬文傑</t>
-  </si>
-  <si>
     <t>陳雅蕾</t>
   </si>
   <si>
@@ -959,9 +941,6 @@
     <t>張秉望</t>
   </si>
   <si>
-    <t>徐    靜</t>
-  </si>
-  <si>
     <t>張祖欣</t>
   </si>
   <si>
@@ -1344,13 +1323,58 @@
   </si>
   <si>
     <t>roll</t>
+  </si>
+  <si>
+    <t>邵麗民</t>
+  </si>
+  <si>
+    <t>涂鳳英</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 黃弘成</t>
+  </si>
+  <si>
+    <t>劉素蘭</t>
+  </si>
+  <si>
+    <t>鄧素珍</t>
+  </si>
+  <si>
+    <t>洪善容</t>
+  </si>
+  <si>
+    <t>熊家緯</t>
+  </si>
+  <si>
+    <t>黃惠美</t>
+  </si>
+  <si>
+    <t>黃惠美看護</t>
+  </si>
+  <si>
+    <t>張淑淨</t>
+  </si>
+  <si>
+    <t>楊曜瑋</t>
+  </si>
+  <si>
+    <t>周傳姜</t>
+  </si>
+  <si>
+    <t>陳羽沛</t>
+  </si>
+  <si>
+    <t>邱慧嫻</t>
+  </si>
+  <si>
+    <t>馬孝政</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1376,12 +1400,6 @@
       <b/>
       <sz val="13"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1431,7 +1449,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1454,13 +1472,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1801,7 +1816,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B436"/>
+  <dimension ref="A1:B444"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="1"/>
   <cols>
     <col min="2" max="2" width="8.77734375" customWidth="1"/>
@@ -1809,10 +1824,10 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.6">
       <c r="A1" s="1" t="s">
-        <v>433</v>
+        <v>426</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>434</v>
+        <v>427</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.6">
@@ -2932,7 +2947,7 @@
     </row>
     <row r="126" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A126" s="5" t="s">
-        <v>124</v>
+        <v>428</v>
       </c>
       <c r="B126" s="3">
         <f t="shared" si="1"/>
@@ -2941,7 +2956,7 @@
     </row>
     <row r="127" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A127" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B127" s="3">
         <f t="shared" si="1"/>
@@ -2950,7 +2965,7 @@
     </row>
     <row r="128" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A128" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B128" s="3">
         <f t="shared" si="1"/>
@@ -2959,7 +2974,7 @@
     </row>
     <row r="129" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A129" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B129" s="3">
         <f t="shared" si="1"/>
@@ -2968,7 +2983,7 @@
     </row>
     <row r="130" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A130" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B130" s="3">
         <f t="shared" si="1"/>
@@ -2977,7 +2992,7 @@
     </row>
     <row r="131" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A131" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B131" s="3">
         <f t="shared" si="1"/>
@@ -2986,7 +3001,7 @@
     </row>
     <row r="132" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A132" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B132" s="3">
         <f t="shared" ref="B132:B195" si="2">B131+1</f>
@@ -2995,7 +3010,7 @@
     </row>
     <row r="133" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A133" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B133" s="3">
         <f t="shared" si="2"/>
@@ -3004,7 +3019,7 @@
     </row>
     <row r="134" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A134" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B134" s="3">
         <f t="shared" si="2"/>
@@ -3013,7 +3028,7 @@
     </row>
     <row r="135" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A135" s="5" t="s">
-        <v>133</v>
+        <v>429</v>
       </c>
       <c r="B135" s="3">
         <f t="shared" si="2"/>
@@ -3022,7 +3037,7 @@
     </row>
     <row r="136" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A136" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B136" s="3">
         <f t="shared" si="2"/>
@@ -3031,7 +3046,7 @@
     </row>
     <row r="137" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A137" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B137" s="3">
         <f t="shared" si="2"/>
@@ -3040,7 +3055,7 @@
     </row>
     <row r="138" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A138" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B138" s="3">
         <f t="shared" si="2"/>
@@ -3049,7 +3064,7 @@
     </row>
     <row r="139" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A139" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B139" s="3">
         <f t="shared" si="2"/>
@@ -3058,7 +3073,7 @@
     </row>
     <row r="140" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A140" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B140" s="3">
         <f t="shared" si="2"/>
@@ -3067,7 +3082,7 @@
     </row>
     <row r="141" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A141" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B141" s="3">
         <f t="shared" si="2"/>
@@ -3076,7 +3091,7 @@
     </row>
     <row r="142" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A142" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B142" s="3">
         <f t="shared" si="2"/>
@@ -3085,7 +3100,7 @@
     </row>
     <row r="143" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A143" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B143" s="3">
         <f t="shared" si="2"/>
@@ -3094,7 +3109,7 @@
     </row>
     <row r="144" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A144" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B144" s="3">
         <f t="shared" si="2"/>
@@ -3103,7 +3118,7 @@
     </row>
     <row r="145" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A145" s="5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B145" s="3">
         <f t="shared" si="2"/>
@@ -3112,7 +3127,7 @@
     </row>
     <row r="146" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A146" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B146" s="3">
         <f t="shared" si="2"/>
@@ -3121,7 +3136,7 @@
     </row>
     <row r="147" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A147" s="5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B147" s="3">
         <f t="shared" si="2"/>
@@ -3130,7 +3145,7 @@
     </row>
     <row r="148" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A148" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B148" s="3">
         <f t="shared" si="2"/>
@@ -3139,7 +3154,7 @@
     </row>
     <row r="149" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A149" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B149" s="3">
         <f t="shared" si="2"/>
@@ -3148,7 +3163,7 @@
     </row>
     <row r="150" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A150" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B150" s="3">
         <f t="shared" si="2"/>
@@ -3157,7 +3172,7 @@
     </row>
     <row r="151" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A151" s="5" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B151" s="3">
         <f t="shared" si="2"/>
@@ -3166,7 +3181,7 @@
     </row>
     <row r="152" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A152" s="5" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B152" s="3">
         <f t="shared" si="2"/>
@@ -3175,7 +3190,7 @@
     </row>
     <row r="153" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A153" s="5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B153" s="3">
         <f t="shared" si="2"/>
@@ -3184,7 +3199,7 @@
     </row>
     <row r="154" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A154" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B154" s="3">
         <f t="shared" si="2"/>
@@ -3193,7 +3208,7 @@
     </row>
     <row r="155" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A155" s="5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B155" s="3">
         <f t="shared" si="2"/>
@@ -3202,7 +3217,7 @@
     </row>
     <row r="156" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A156" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B156" s="3">
         <f t="shared" si="2"/>
@@ -3211,7 +3226,7 @@
     </row>
     <row r="157" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A157" s="5" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B157" s="3">
         <f t="shared" si="2"/>
@@ -3220,7 +3235,7 @@
     </row>
     <row r="158" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A158" s="5" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B158" s="3">
         <f t="shared" si="2"/>
@@ -3229,7 +3244,7 @@
     </row>
     <row r="159" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A159" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B159" s="3">
         <f t="shared" si="2"/>
@@ -3238,7 +3253,7 @@
     </row>
     <row r="160" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A160" s="5" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B160" s="3">
         <f t="shared" si="2"/>
@@ -3247,7 +3262,7 @@
     </row>
     <row r="161" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A161" s="5" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B161" s="3">
         <f t="shared" si="2"/>
@@ -3256,7 +3271,7 @@
     </row>
     <row r="162" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A162" s="5" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B162" s="3">
         <f t="shared" si="2"/>
@@ -3265,7 +3280,7 @@
     </row>
     <row r="163" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A163" s="5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B163" s="3">
         <f t="shared" si="2"/>
@@ -3274,7 +3289,7 @@
     </row>
     <row r="164" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A164" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B164" s="3">
         <f t="shared" si="2"/>
@@ -3283,7 +3298,7 @@
     </row>
     <row r="165" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A165" s="5" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B165" s="3">
         <f t="shared" si="2"/>
@@ -3292,7 +3307,7 @@
     </row>
     <row r="166" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A166" s="5" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B166" s="3">
         <f t="shared" si="2"/>
@@ -3301,7 +3316,7 @@
     </row>
     <row r="167" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A167" s="5" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B167" s="3">
         <f t="shared" si="2"/>
@@ -3310,7 +3325,7 @@
     </row>
     <row r="168" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A168" s="5" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B168" s="3">
         <f t="shared" si="2"/>
@@ -3319,7 +3334,7 @@
     </row>
     <row r="169" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A169" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B169" s="3">
         <f t="shared" si="2"/>
@@ -3328,7 +3343,7 @@
     </row>
     <row r="170" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A170" s="5" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B170" s="3">
         <f t="shared" si="2"/>
@@ -3337,7 +3352,7 @@
     </row>
     <row r="171" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A171" s="5" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B171" s="3">
         <f t="shared" si="2"/>
@@ -3346,7 +3361,7 @@
     </row>
     <row r="172" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A172" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B172" s="3">
         <f t="shared" si="2"/>
@@ -3355,7 +3370,7 @@
     </row>
     <row r="173" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A173" s="5" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B173" s="3">
         <f t="shared" si="2"/>
@@ -3364,7 +3379,7 @@
     </row>
     <row r="174" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A174" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B174" s="3">
         <f t="shared" si="2"/>
@@ -3373,7 +3388,7 @@
     </row>
     <row r="175" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A175" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B175" s="3">
         <f t="shared" si="2"/>
@@ -3382,7 +3397,7 @@
     </row>
     <row r="176" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A176" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B176" s="3">
         <f t="shared" si="2"/>
@@ -3391,7 +3406,7 @@
     </row>
     <row r="177" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A177" s="5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B177" s="3">
         <f t="shared" si="2"/>
@@ -3400,7 +3415,7 @@
     </row>
     <row r="178" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A178" s="5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B178" s="3">
         <f t="shared" si="2"/>
@@ -3409,7 +3424,7 @@
     </row>
     <row r="179" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A179" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B179" s="3">
         <f t="shared" si="2"/>
@@ -3418,7 +3433,7 @@
     </row>
     <row r="180" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A180" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B180" s="3">
         <f t="shared" si="2"/>
@@ -3427,7 +3442,7 @@
     </row>
     <row r="181" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A181" s="5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B181" s="3">
         <f t="shared" si="2"/>
@@ -3436,7 +3451,7 @@
     </row>
     <row r="182" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A182" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B182" s="3">
         <f t="shared" si="2"/>
@@ -3445,7 +3460,7 @@
     </row>
     <row r="183" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A183" s="5" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B183" s="3">
         <f t="shared" si="2"/>
@@ -3454,7 +3469,7 @@
     </row>
     <row r="184" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A184" s="5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B184" s="3">
         <f t="shared" si="2"/>
@@ -3463,7 +3478,7 @@
     </row>
     <row r="185" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A185" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B185" s="3">
         <f t="shared" si="2"/>
@@ -3472,7 +3487,7 @@
     </row>
     <row r="186" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A186" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B186" s="3">
         <f t="shared" si="2"/>
@@ -3481,7 +3496,7 @@
     </row>
     <row r="187" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A187" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B187" s="3">
         <f t="shared" si="2"/>
@@ -3490,7 +3505,7 @@
     </row>
     <row r="188" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A188" s="5" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B188" s="3">
         <f t="shared" si="2"/>
@@ -3499,7 +3514,7 @@
     </row>
     <row r="189" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A189" s="5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B189" s="3">
         <f t="shared" si="2"/>
@@ -3508,7 +3523,7 @@
     </row>
     <row r="190" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A190" s="5" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B190" s="3">
         <f t="shared" si="2"/>
@@ -3517,7 +3532,7 @@
     </row>
     <row r="191" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A191" s="5" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B191" s="3">
         <f t="shared" si="2"/>
@@ -3526,7 +3541,7 @@
     </row>
     <row r="192" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A192" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B192" s="3">
         <f t="shared" si="2"/>
@@ -3535,7 +3550,7 @@
     </row>
     <row r="193" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A193" s="5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B193" s="3">
         <f t="shared" si="2"/>
@@ -3544,7 +3559,7 @@
     </row>
     <row r="194" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A194" s="5" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B194" s="3">
         <f t="shared" si="2"/>
@@ -3553,7 +3568,7 @@
     </row>
     <row r="195" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A195" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B195" s="3">
         <f t="shared" si="2"/>
@@ -3562,7 +3577,7 @@
     </row>
     <row r="196" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A196" s="5" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B196" s="3">
         <f t="shared" ref="B196:B259" si="3">B195+1</f>
@@ -3571,7 +3586,7 @@
     </row>
     <row r="197" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A197" s="5" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B197" s="3">
         <f t="shared" si="3"/>
@@ -3580,7 +3595,7 @@
     </row>
     <row r="198" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A198" s="5" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B198" s="3">
         <f t="shared" si="3"/>
@@ -3589,7 +3604,7 @@
     </row>
     <row r="199" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A199" s="5" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B199" s="3">
         <f t="shared" si="3"/>
@@ -3598,7 +3613,7 @@
     </row>
     <row r="200" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A200" s="5" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B200" s="3">
         <f t="shared" si="3"/>
@@ -3607,7 +3622,7 @@
     </row>
     <row r="201" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A201" s="7" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B201" s="3">
         <f t="shared" si="3"/>
@@ -3616,7 +3631,7 @@
     </row>
     <row r="202" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A202" s="7" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B202" s="3">
         <f t="shared" si="3"/>
@@ -3625,7 +3640,7 @@
     </row>
     <row r="203" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A203" s="7" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B203" s="3">
         <f t="shared" si="3"/>
@@ -3634,7 +3649,7 @@
     </row>
     <row r="204" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A204" s="7" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B204" s="3">
         <f t="shared" si="3"/>
@@ -3643,7 +3658,7 @@
     </row>
     <row r="205" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A205" s="7" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B205" s="3">
         <f t="shared" si="3"/>
@@ -3652,7 +3667,7 @@
     </row>
     <row r="206" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A206" s="7" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B206" s="3">
         <f t="shared" si="3"/>
@@ -3661,7 +3676,7 @@
     </row>
     <row r="207" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A207" s="7" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B207" s="3">
         <f t="shared" si="3"/>
@@ -3670,7 +3685,7 @@
     </row>
     <row r="208" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A208" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B208" s="3">
         <f t="shared" si="3"/>
@@ -3679,7 +3694,7 @@
     </row>
     <row r="209" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A209" s="7" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B209" s="3">
         <f t="shared" si="3"/>
@@ -3688,7 +3703,7 @@
     </row>
     <row r="210" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A210" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B210" s="3">
         <f t="shared" si="3"/>
@@ -3697,7 +3712,7 @@
     </row>
     <row r="211" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A211" s="7" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B211" s="3">
         <f t="shared" si="3"/>
@@ -3706,7 +3721,7 @@
     </row>
     <row r="212" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A212" s="7" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B212" s="3">
         <f t="shared" si="3"/>
@@ -3715,7 +3730,7 @@
     </row>
     <row r="213" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A213" s="7" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B213" s="3">
         <f t="shared" si="3"/>
@@ -3724,7 +3739,7 @@
     </row>
     <row r="214" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A214" s="7" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B214" s="3">
         <f t="shared" si="3"/>
@@ -3733,7 +3748,7 @@
     </row>
     <row r="215" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A215" s="7" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B215" s="3">
         <f t="shared" si="3"/>
@@ -3742,7 +3757,7 @@
     </row>
     <row r="216" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A216" s="7" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B216" s="3">
         <f t="shared" si="3"/>
@@ -3751,7 +3766,7 @@
     </row>
     <row r="217" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A217" s="7" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B217" s="3">
         <f t="shared" si="3"/>
@@ -3760,7 +3775,7 @@
     </row>
     <row r="218" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A218" s="7" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B218" s="3">
         <f t="shared" si="3"/>
@@ -3769,7 +3784,7 @@
     </row>
     <row r="219" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A219" s="7" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B219" s="3">
         <f t="shared" si="3"/>
@@ -3778,7 +3793,7 @@
     </row>
     <row r="220" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A220" s="7" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B220" s="3">
         <f t="shared" si="3"/>
@@ -3787,7 +3802,7 @@
     </row>
     <row r="221" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A221" s="7" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B221" s="3">
         <f t="shared" si="3"/>
@@ -3796,25 +3811,25 @@
     </row>
     <row r="222" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A222" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="B222" s="3">
+        <f t="shared" si="3"/>
+        <v>221</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" ht="15.6" outlineLevel="1">
+      <c r="A223" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="B223" s="3">
+        <f t="shared" si="3"/>
+        <v>222</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" ht="15.6" outlineLevel="1">
+      <c r="A224" s="7" t="s">
         <v>220</v>
-      </c>
-      <c r="B222" s="3">
-        <f t="shared" si="3"/>
-        <v>221</v>
-      </c>
-    </row>
-    <row r="223" spans="1:2" ht="15.6" outlineLevel="1">
-      <c r="A223" s="8" t="s">
-        <v>221</v>
-      </c>
-      <c r="B223" s="3">
-        <f t="shared" si="3"/>
-        <v>222</v>
-      </c>
-    </row>
-    <row r="224" spans="1:2" ht="15.6" outlineLevel="1">
-      <c r="A224" s="8" t="s">
-        <v>222</v>
       </c>
       <c r="B224" s="3">
         <f t="shared" si="3"/>
@@ -3823,7 +3838,7 @@
     </row>
     <row r="225" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A225" s="7" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B225" s="3">
         <f t="shared" si="3"/>
@@ -3832,7 +3847,7 @@
     </row>
     <row r="226" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A226" s="7" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B226" s="3">
         <f t="shared" si="3"/>
@@ -3841,7 +3856,7 @@
     </row>
     <row r="227" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A227" s="7" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B227" s="3">
         <f t="shared" si="3"/>
@@ -3850,7 +3865,7 @@
     </row>
     <row r="228" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A228" s="7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B228" s="3">
         <f t="shared" si="3"/>
@@ -3859,7 +3874,7 @@
     </row>
     <row r="229" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A229" s="7" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B229" s="3">
         <f t="shared" si="3"/>
@@ -3868,7 +3883,7 @@
     </row>
     <row r="230" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A230" s="7" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B230" s="3">
         <f t="shared" si="3"/>
@@ -3877,7 +3892,7 @@
     </row>
     <row r="231" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A231" s="7" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B231" s="3">
         <f t="shared" si="3"/>
@@ -3886,7 +3901,7 @@
     </row>
     <row r="232" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A232" s="7" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B232" s="3">
         <f t="shared" si="3"/>
@@ -3895,7 +3910,7 @@
     </row>
     <row r="233" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A233" s="7" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B233" s="3">
         <f t="shared" si="3"/>
@@ -3904,7 +3919,7 @@
     </row>
     <row r="234" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A234" s="7" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B234" s="3">
         <f t="shared" si="3"/>
@@ -3913,7 +3928,7 @@
     </row>
     <row r="235" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A235" s="7" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B235" s="3">
         <f t="shared" si="3"/>
@@ -3922,7 +3937,7 @@
     </row>
     <row r="236" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A236" s="7" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B236" s="3">
         <f t="shared" si="3"/>
@@ -3931,7 +3946,7 @@
     </row>
     <row r="237" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A237" s="7" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B237" s="3">
         <f t="shared" si="3"/>
@@ -3940,7 +3955,7 @@
     </row>
     <row r="238" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A238" s="7" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B238" s="3">
         <f t="shared" si="3"/>
@@ -3949,7 +3964,7 @@
     </row>
     <row r="239" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A239" s="7" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B239" s="3">
         <f t="shared" si="3"/>
@@ -3958,7 +3973,7 @@
     </row>
     <row r="240" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A240" s="7" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B240" s="3">
         <f t="shared" si="3"/>
@@ -3967,7 +3982,7 @@
     </row>
     <row r="241" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A241" s="7" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B241" s="3">
         <f t="shared" si="3"/>
@@ -3976,7 +3991,7 @@
     </row>
     <row r="242" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A242" s="7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B242" s="3">
         <f t="shared" si="3"/>
@@ -3985,7 +4000,7 @@
     </row>
     <row r="243" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A243" s="7" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B243" s="3">
         <f t="shared" si="3"/>
@@ -3994,7 +4009,7 @@
     </row>
     <row r="244" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A244" s="7" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B244" s="3">
         <f t="shared" si="3"/>
@@ -4003,7 +4018,7 @@
     </row>
     <row r="245" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A245" s="7" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B245" s="3">
         <f t="shared" si="3"/>
@@ -4012,7 +4027,7 @@
     </row>
     <row r="246" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A246" s="7" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B246" s="3">
         <f t="shared" si="3"/>
@@ -4021,7 +4036,7 @@
     </row>
     <row r="247" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A247" s="7" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B247" s="3">
         <f t="shared" si="3"/>
@@ -4030,7 +4045,7 @@
     </row>
     <row r="248" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A248" s="7" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B248" s="3">
         <f t="shared" si="3"/>
@@ -4039,7 +4054,7 @@
     </row>
     <row r="249" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A249" s="7" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B249" s="3">
         <f t="shared" si="3"/>
@@ -4048,7 +4063,7 @@
     </row>
     <row r="250" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A250" s="7" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B250" s="3">
         <f t="shared" si="3"/>
@@ -4057,7 +4072,7 @@
     </row>
     <row r="251" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A251" s="7" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B251" s="3">
         <f t="shared" si="3"/>
@@ -4066,7 +4081,7 @@
     </row>
     <row r="252" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A252" s="7" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B252" s="3">
         <f t="shared" si="3"/>
@@ -4075,7 +4090,7 @@
     </row>
     <row r="253" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A253" s="7" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B253" s="3">
         <f t="shared" si="3"/>
@@ -4084,7 +4099,7 @@
     </row>
     <row r="254" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A254" s="7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B254" s="3">
         <f t="shared" si="3"/>
@@ -4093,7 +4108,7 @@
     </row>
     <row r="255" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A255" s="7" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B255" s="3">
         <f t="shared" si="3"/>
@@ -4102,7 +4117,7 @@
     </row>
     <row r="256" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A256" s="7" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B256" s="3">
         <f t="shared" si="3"/>
@@ -4111,7 +4126,7 @@
     </row>
     <row r="257" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A257" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B257" s="3">
         <f t="shared" si="3"/>
@@ -4120,7 +4135,7 @@
     </row>
     <row r="258" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A258" s="7" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B258" s="3">
         <f t="shared" si="3"/>
@@ -4129,7 +4144,7 @@
     </row>
     <row r="259" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A259" s="7" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B259" s="3">
         <f t="shared" si="3"/>
@@ -4138,7 +4153,7 @@
     </row>
     <row r="260" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A260" s="7" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B260" s="3">
         <f t="shared" ref="B260:B323" si="4">B259+1</f>
@@ -4147,7 +4162,7 @@
     </row>
     <row r="261" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A261" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B261" s="3">
         <f t="shared" si="4"/>
@@ -4156,7 +4171,7 @@
     </row>
     <row r="262" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A262" s="7" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B262" s="3">
         <f t="shared" si="4"/>
@@ -4165,7 +4180,7 @@
     </row>
     <row r="263" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A263" s="7" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B263" s="3">
         <f t="shared" si="4"/>
@@ -4174,7 +4189,7 @@
     </row>
     <row r="264" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A264" s="7" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B264" s="3">
         <f t="shared" si="4"/>
@@ -4183,7 +4198,7 @@
     </row>
     <row r="265" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A265" s="7" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B265" s="3">
         <f t="shared" si="4"/>
@@ -4192,34 +4207,34 @@
     </row>
     <row r="266" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A266" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="B266" s="3">
+        <f t="shared" si="4"/>
+        <v>265</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2" ht="15.6" outlineLevel="1">
+      <c r="A267" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="B267" s="3">
+        <f t="shared" si="4"/>
+        <v>266</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2" ht="15.6" outlineLevel="1">
+      <c r="A268" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="B266" s="3">
-        <f t="shared" si="4"/>
+      <c r="B268" s="3">
+        <f t="shared" si="4"/>
+        <v>267</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2" ht="15.6" outlineLevel="1">
+      <c r="A269" s="5" t="s">
         <v>265</v>
-      </c>
-    </row>
-    <row r="267" spans="1:2" ht="15.6" outlineLevel="1">
-      <c r="A267" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="B267" s="3">
-        <f t="shared" si="4"/>
-        <v>266</v>
-      </c>
-    </row>
-    <row r="268" spans="1:2" ht="15.6" outlineLevel="1">
-      <c r="A268" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="B268" s="3">
-        <f t="shared" si="4"/>
-        <v>267</v>
-      </c>
-    </row>
-    <row r="269" spans="1:2" ht="15.6" outlineLevel="1">
-      <c r="A269" s="7" t="s">
-        <v>267</v>
       </c>
       <c r="B269" s="3">
         <f t="shared" si="4"/>
@@ -4228,7 +4243,7 @@
     </row>
     <row r="270" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A270" s="5" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B270" s="3">
         <f t="shared" si="4"/>
@@ -4237,7 +4252,7 @@
     </row>
     <row r="271" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A271" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B271" s="3">
         <f t="shared" si="4"/>
@@ -4246,7 +4261,7 @@
     </row>
     <row r="272" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A272" s="5" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B272" s="3">
         <f t="shared" si="4"/>
@@ -4255,7 +4270,7 @@
     </row>
     <row r="273" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A273" s="5" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B273" s="3">
         <f t="shared" si="4"/>
@@ -4264,7 +4279,7 @@
     </row>
     <row r="274" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A274" s="5" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B274" s="3">
         <f t="shared" si="4"/>
@@ -4273,7 +4288,7 @@
     </row>
     <row r="275" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A275" s="5" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B275" s="3">
         <f t="shared" si="4"/>
@@ -4282,7 +4297,7 @@
     </row>
     <row r="276" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A276" s="5" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B276" s="3">
         <f t="shared" si="4"/>
@@ -4291,7 +4306,7 @@
     </row>
     <row r="277" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A277" s="5" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B277" s="3">
         <f t="shared" si="4"/>
@@ -4300,7 +4315,7 @@
     </row>
     <row r="278" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A278" s="5" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B278" s="3">
         <f t="shared" si="4"/>
@@ -4309,7 +4324,7 @@
     </row>
     <row r="279" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A279" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B279" s="3">
         <f t="shared" si="4"/>
@@ -4318,7 +4333,7 @@
     </row>
     <row r="280" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A280" s="5" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B280" s="3">
         <f t="shared" si="4"/>
@@ -4327,7 +4342,7 @@
     </row>
     <row r="281" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A281" s="5" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B281" s="3">
         <f t="shared" si="4"/>
@@ -4336,7 +4351,7 @@
     </row>
     <row r="282" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A282" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B282" s="3">
         <f t="shared" si="4"/>
@@ -4345,7 +4360,7 @@
     </row>
     <row r="283" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A283" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B283" s="3">
         <f t="shared" si="4"/>
@@ -4354,7 +4369,7 @@
     </row>
     <row r="284" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A284" s="5" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B284" s="3">
         <f t="shared" si="4"/>
@@ -4363,7 +4378,7 @@
     </row>
     <row r="285" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A285" s="5" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B285" s="3">
         <f t="shared" si="4"/>
@@ -4372,34 +4387,34 @@
     </row>
     <row r="286" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A286" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="B286" s="3">
+        <f t="shared" si="4"/>
+        <v>285</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2" ht="15.6" outlineLevel="1">
+      <c r="A287" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="B287" s="3">
+        <f t="shared" si="4"/>
+        <v>286</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2" ht="15.6" outlineLevel="1">
+      <c r="A288" s="7" t="s">
         <v>284</v>
       </c>
-      <c r="B286" s="3">
-        <f t="shared" si="4"/>
+      <c r="B288" s="3">
+        <f t="shared" si="4"/>
+        <v>287</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2" ht="15.6" outlineLevel="1">
+      <c r="A289" s="7" t="s">
         <v>285</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2" ht="15.6" outlineLevel="1">
-      <c r="A287" s="5" t="s">
-        <v>285</v>
-      </c>
-      <c r="B287" s="3">
-        <f t="shared" si="4"/>
-        <v>286</v>
-      </c>
-    </row>
-    <row r="288" spans="1:2" ht="15.6" outlineLevel="1">
-      <c r="A288" s="5" t="s">
-        <v>286</v>
-      </c>
-      <c r="B288" s="3">
-        <f t="shared" si="4"/>
-        <v>287</v>
-      </c>
-    </row>
-    <row r="289" spans="1:2" ht="15.6" outlineLevel="1">
-      <c r="A289" s="5" t="s">
-        <v>287</v>
       </c>
       <c r="B289" s="3">
         <f t="shared" si="4"/>
@@ -4408,7 +4423,7 @@
     </row>
     <row r="290" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A290" s="7" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B290" s="3">
         <f t="shared" si="4"/>
@@ -4417,7 +4432,7 @@
     </row>
     <row r="291" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A291" s="7" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B291" s="3">
         <f t="shared" si="4"/>
@@ -4426,7 +4441,7 @@
     </row>
     <row r="292" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A292" s="7" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B292" s="3">
         <f t="shared" si="4"/>
@@ -4435,7 +4450,7 @@
     </row>
     <row r="293" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A293" s="7" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B293" s="3">
         <f t="shared" si="4"/>
@@ -4444,7 +4459,7 @@
     </row>
     <row r="294" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A294" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B294" s="3">
         <f t="shared" si="4"/>
@@ -4453,7 +4468,7 @@
     </row>
     <row r="295" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A295" s="7" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B295" s="3">
         <f t="shared" si="4"/>
@@ -4462,7 +4477,7 @@
     </row>
     <row r="296" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A296" s="7" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B296" s="3">
         <f t="shared" si="4"/>
@@ -4471,43 +4486,43 @@
     </row>
     <row r="297" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A297" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="B297" s="3">
+        <f t="shared" si="4"/>
+        <v>296</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2" ht="15.6" outlineLevel="1">
+      <c r="A298" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="B298" s="3">
+        <f t="shared" si="4"/>
+        <v>297</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2" ht="15.6" outlineLevel="1">
+      <c r="A299" s="5" t="s">
         <v>295</v>
       </c>
-      <c r="B297" s="3">
-        <f t="shared" si="4"/>
+      <c r="B299" s="3">
+        <f t="shared" si="4"/>
+        <v>298</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" ht="17.25" customHeight="1" outlineLevel="1">
+      <c r="A300" s="5" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="298" spans="1:2" ht="15.6" outlineLevel="1">
-      <c r="A298" s="7" t="s">
-        <v>296</v>
-      </c>
-      <c r="B298" s="3">
-        <f t="shared" si="4"/>
+      <c r="B300" s="3">
+        <f t="shared" si="4"/>
+        <v>299</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2" ht="17.25" customHeight="1" outlineLevel="1">
+      <c r="A301" s="5" t="s">
         <v>297</v>
-      </c>
-    </row>
-    <row r="299" spans="1:2" ht="15.6" outlineLevel="1">
-      <c r="A299" s="7" t="s">
-        <v>297</v>
-      </c>
-      <c r="B299" s="3">
-        <f t="shared" si="4"/>
-        <v>298</v>
-      </c>
-    </row>
-    <row r="300" spans="1:2" ht="17.25" customHeight="1" outlineLevel="1">
-      <c r="A300" s="7" t="s">
-        <v>298</v>
-      </c>
-      <c r="B300" s="3">
-        <f t="shared" si="4"/>
-        <v>299</v>
-      </c>
-    </row>
-    <row r="301" spans="1:2" ht="17.25" customHeight="1" outlineLevel="1">
-      <c r="A301" s="7" t="s">
-        <v>299</v>
       </c>
       <c r="B301" s="3">
         <f t="shared" si="4"/>
@@ -4516,7 +4531,7 @@
     </row>
     <row r="302" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A302" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B302" s="3">
         <f t="shared" si="4"/>
@@ -4525,7 +4540,7 @@
     </row>
     <row r="303" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A303" s="5" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B303" s="3">
         <f t="shared" si="4"/>
@@ -4534,7 +4549,7 @@
     </row>
     <row r="304" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A304" s="5" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B304" s="3">
         <f t="shared" si="4"/>
@@ -4543,7 +4558,7 @@
     </row>
     <row r="305" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A305" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B305" s="3">
         <f t="shared" si="4"/>
@@ -4552,7 +4567,7 @@
     </row>
     <row r="306" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A306" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B306" s="3">
         <f t="shared" si="4"/>
@@ -4561,7 +4576,7 @@
     </row>
     <row r="307" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A307" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B307" s="3">
         <f t="shared" si="4"/>
@@ -4570,7 +4585,7 @@
     </row>
     <row r="308" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A308" s="5" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B308" s="3">
         <f t="shared" si="4"/>
@@ -4579,7 +4594,7 @@
     </row>
     <row r="309" spans="1:2" ht="15.6">
       <c r="A309" s="5" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="B309" s="3">
         <f t="shared" si="4"/>
@@ -4588,7 +4603,7 @@
     </row>
     <row r="310" spans="1:2" ht="15.6">
       <c r="A310" s="5" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B310" s="3">
         <f t="shared" si="4"/>
@@ -4597,7 +4612,7 @@
     </row>
     <row r="311" spans="1:2" ht="15.6">
       <c r="A311" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B311" s="3">
         <f t="shared" si="4"/>
@@ -4606,7 +4621,7 @@
     </row>
     <row r="312" spans="1:2" ht="15.6">
       <c r="A312" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B312" s="3">
         <f t="shared" si="4"/>
@@ -4615,7 +4630,7 @@
     </row>
     <row r="313" spans="1:2" ht="15.6">
       <c r="A313" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B313" s="3">
         <f t="shared" si="4"/>
@@ -4624,7 +4639,7 @@
     </row>
     <row r="314" spans="1:2" ht="15.6">
       <c r="A314" s="5" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B314" s="3">
         <f t="shared" si="4"/>
@@ -4633,7 +4648,7 @@
     </row>
     <row r="315" spans="1:2" ht="15.6">
       <c r="A315" s="5" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B315" s="3">
         <f t="shared" si="4"/>
@@ -4641,8 +4656,8 @@
       </c>
     </row>
     <row r="316" spans="1:2" ht="15.6">
-      <c r="A316" s="5" t="s">
-        <v>314</v>
+      <c r="A316" s="8" t="s">
+        <v>312</v>
       </c>
       <c r="B316" s="3">
         <f t="shared" si="4"/>
@@ -4651,7 +4666,7 @@
     </row>
     <row r="317" spans="1:2" ht="15.6">
       <c r="A317" s="5" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B317" s="3">
         <f t="shared" si="4"/>
@@ -4660,7 +4675,7 @@
     </row>
     <row r="318" spans="1:2" ht="15.6">
       <c r="A318" s="5" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B318" s="3">
         <f t="shared" si="4"/>
@@ -4669,7 +4684,7 @@
     </row>
     <row r="319" spans="1:2" ht="15.6">
       <c r="A319" s="5" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B319" s="3">
         <f t="shared" si="4"/>
@@ -4678,7 +4693,7 @@
     </row>
     <row r="320" spans="1:2" ht="15.6">
       <c r="A320" s="5" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B320" s="3">
         <f t="shared" si="4"/>
@@ -4686,8 +4701,8 @@
       </c>
     </row>
     <row r="321" spans="1:2" ht="15.6">
-      <c r="A321" s="9" t="s">
-        <v>319</v>
+      <c r="A321" s="5" t="s">
+        <v>317</v>
       </c>
       <c r="B321" s="3">
         <f t="shared" si="4"/>
@@ -4696,25 +4711,25 @@
     </row>
     <row r="322" spans="1:2" ht="15.6">
       <c r="A322" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="B322" s="3">
+        <f t="shared" si="4"/>
+        <v>321</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2" ht="15.6">
+      <c r="A323" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="B323" s="3">
+        <f t="shared" si="4"/>
+        <v>322</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2" ht="15.6">
+      <c r="A324" s="7" t="s">
         <v>320</v>
-      </c>
-      <c r="B322" s="3">
-        <f t="shared" si="4"/>
-        <v>321</v>
-      </c>
-    </row>
-    <row r="323" spans="1:2" ht="15.6">
-      <c r="A323" s="5" t="s">
-        <v>321</v>
-      </c>
-      <c r="B323" s="3">
-        <f t="shared" si="4"/>
-        <v>322</v>
-      </c>
-    </row>
-    <row r="324" spans="1:2" ht="15.6">
-      <c r="A324" s="5" t="s">
-        <v>322</v>
       </c>
       <c r="B324" s="3">
         <f t="shared" ref="B324:B387" si="5">B323+1</f>
@@ -4723,25 +4738,25 @@
     </row>
     <row r="325" spans="1:2" ht="17.25" customHeight="1">
       <c r="A325" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="B325" s="3">
+        <f t="shared" si="5"/>
+        <v>324</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A326" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="B326" s="3">
+        <f t="shared" si="5"/>
+        <v>325</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A327" s="7" t="s">
         <v>323</v>
-      </c>
-      <c r="B325" s="3">
-        <f t="shared" si="5"/>
-        <v>324</v>
-      </c>
-    </row>
-    <row r="326" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A326" s="5" t="s">
-        <v>324</v>
-      </c>
-      <c r="B326" s="3">
-        <f t="shared" si="5"/>
-        <v>325</v>
-      </c>
-    </row>
-    <row r="327" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A327" s="5" t="s">
-        <v>325</v>
       </c>
       <c r="B327" s="3">
         <f t="shared" si="5"/>
@@ -4750,7 +4765,7 @@
     </row>
     <row r="328" spans="1:2" ht="17.25" customHeight="1">
       <c r="A328" s="7" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B328" s="3">
         <f t="shared" si="5"/>
@@ -4759,7 +4774,7 @@
     </row>
     <row r="329" spans="1:2" ht="17.25" customHeight="1">
       <c r="A329" s="7" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B329" s="3">
         <f t="shared" si="5"/>
@@ -4768,25 +4783,25 @@
     </row>
     <row r="330" spans="1:2" ht="15.6">
       <c r="A330" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="B330" s="3">
+        <f t="shared" si="5"/>
+        <v>329</v>
+      </c>
+    </row>
+    <row r="331" spans="1:2" ht="15.6">
+      <c r="A331" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="B331" s="3">
+        <f t="shared" si="5"/>
+        <v>330</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2" ht="15.6">
+      <c r="A332" s="5" t="s">
         <v>328</v>
-      </c>
-      <c r="B330" s="3">
-        <f t="shared" si="5"/>
-        <v>329</v>
-      </c>
-    </row>
-    <row r="331" spans="1:2" ht="15.6">
-      <c r="A331" s="7" t="s">
-        <v>329</v>
-      </c>
-      <c r="B331" s="3">
-        <f t="shared" si="5"/>
-        <v>330</v>
-      </c>
-    </row>
-    <row r="332" spans="1:2" ht="15.6">
-      <c r="A332" s="7" t="s">
-        <v>330</v>
       </c>
       <c r="B332" s="3">
         <f t="shared" si="5"/>
@@ -4795,7 +4810,7 @@
     </row>
     <row r="333" spans="1:2" ht="15.6">
       <c r="A333" s="7" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B333" s="3">
         <f t="shared" si="5"/>
@@ -4804,34 +4819,34 @@
     </row>
     <row r="334" spans="1:2" ht="15.6">
       <c r="A334" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="B334" s="3">
+        <f t="shared" si="5"/>
+        <v>333</v>
+      </c>
+    </row>
+    <row r="335" spans="1:2" ht="15.6">
+      <c r="A335" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="B335" s="3">
+        <f t="shared" si="5"/>
+        <v>334</v>
+      </c>
+    </row>
+    <row r="336" spans="1:2" ht="15.6">
+      <c r="A336" s="7" t="s">
         <v>332</v>
       </c>
-      <c r="B334" s="3">
-        <f t="shared" si="5"/>
+      <c r="B336" s="3">
+        <f t="shared" si="5"/>
+        <v>335</v>
+      </c>
+    </row>
+    <row r="337" spans="1:2" ht="15.6">
+      <c r="A337" s="7" t="s">
         <v>333</v>
-      </c>
-    </row>
-    <row r="335" spans="1:2" ht="15.6">
-      <c r="A335" s="5" t="s">
-        <v>333</v>
-      </c>
-      <c r="B335" s="3">
-        <f t="shared" si="5"/>
-        <v>334</v>
-      </c>
-    </row>
-    <row r="336" spans="1:2" ht="15.6">
-      <c r="A336" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="B336" s="3">
-        <f t="shared" si="5"/>
-        <v>335</v>
-      </c>
-    </row>
-    <row r="337" spans="1:2" ht="15.6">
-      <c r="A337" s="5" t="s">
-        <v>335</v>
       </c>
       <c r="B337" s="3">
         <f t="shared" si="5"/>
@@ -4840,7 +4855,7 @@
     </row>
     <row r="338" spans="1:2" ht="15.6">
       <c r="A338" s="7" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B338" s="3">
         <f t="shared" si="5"/>
@@ -4849,7 +4864,7 @@
     </row>
     <row r="339" spans="1:2" ht="15.6">
       <c r="A339" s="7" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B339" s="3">
         <f t="shared" si="5"/>
@@ -4858,7 +4873,7 @@
     </row>
     <row r="340" spans="1:2" ht="15.6">
       <c r="A340" s="7" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B340" s="3">
         <f t="shared" si="5"/>
@@ -4867,7 +4882,7 @@
     </row>
     <row r="341" spans="1:2" ht="15.6">
       <c r="A341" s="7" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B341" s="3">
         <f t="shared" si="5"/>
@@ -4876,25 +4891,25 @@
     </row>
     <row r="342" spans="1:2" ht="15.6">
       <c r="A342" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="B342" s="3">
+        <f t="shared" si="5"/>
+        <v>341</v>
+      </c>
+    </row>
+    <row r="343" spans="1:2" ht="15.6">
+      <c r="A343" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="B343" s="3">
+        <f t="shared" si="5"/>
+        <v>342</v>
+      </c>
+    </row>
+    <row r="344" spans="1:2" ht="15.6">
+      <c r="A344" s="9" t="s">
         <v>340</v>
-      </c>
-      <c r="B342" s="3">
-        <f t="shared" si="5"/>
-        <v>341</v>
-      </c>
-    </row>
-    <row r="343" spans="1:2" ht="15.6">
-      <c r="A343" s="7" t="s">
-        <v>341</v>
-      </c>
-      <c r="B343" s="3">
-        <f t="shared" si="5"/>
-        <v>342</v>
-      </c>
-    </row>
-    <row r="344" spans="1:2" ht="15.6">
-      <c r="A344" s="7" t="s">
-        <v>342</v>
       </c>
       <c r="B344" s="3">
         <f t="shared" si="5"/>
@@ -4903,7 +4918,7 @@
     </row>
     <row r="345" spans="1:2" ht="15.6">
       <c r="A345" s="7" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B345" s="3">
         <f t="shared" si="5"/>
@@ -4912,7 +4927,7 @@
     </row>
     <row r="346" spans="1:2" ht="15.6">
       <c r="A346" s="7" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B346" s="3">
         <f t="shared" si="5"/>
@@ -4921,61 +4936,61 @@
     </row>
     <row r="347" spans="1:2" ht="15.6">
       <c r="A347" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="B347" s="3">
+        <f t="shared" si="5"/>
+        <v>346</v>
+      </c>
+    </row>
+    <row r="348" spans="1:2" ht="15.6">
+      <c r="A348" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="B348" s="3">
+        <f t="shared" si="5"/>
+        <v>347</v>
+      </c>
+    </row>
+    <row r="349" spans="1:2" ht="15.6">
+      <c r="A349" s="4" t="s">
         <v>345</v>
       </c>
-      <c r="B347" s="3">
-        <f t="shared" si="5"/>
+      <c r="B349" s="3">
+        <f t="shared" si="5"/>
+        <v>348</v>
+      </c>
+    </row>
+    <row r="350" spans="1:2" ht="15.6">
+      <c r="A350" s="4" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="348" spans="1:2" ht="15.6">
-      <c r="A348" s="10" t="s">
-        <v>346</v>
-      </c>
-      <c r="B348" s="3">
-        <f t="shared" si="5"/>
+      <c r="B350" s="3">
+        <f t="shared" si="5"/>
+        <v>349</v>
+      </c>
+    </row>
+    <row r="351" spans="1:2" ht="15.6">
+      <c r="A351" s="4" t="s">
         <v>347</v>
       </c>
-    </row>
-    <row r="349" spans="1:2" ht="15.6">
-      <c r="A349" s="10" t="s">
-        <v>347</v>
-      </c>
-      <c r="B349" s="3">
-        <f t="shared" si="5"/>
+      <c r="B351" s="3">
+        <f t="shared" si="5"/>
+        <v>350</v>
+      </c>
+    </row>
+    <row r="352" spans="1:2" ht="15.6">
+      <c r="A352" s="4" t="s">
         <v>348</v>
       </c>
-    </row>
-    <row r="350" spans="1:2" ht="15.6">
-      <c r="A350" s="7" t="s">
-        <v>348</v>
-      </c>
-      <c r="B350" s="3">
-        <f t="shared" si="5"/>
+      <c r="B352" s="3">
+        <f t="shared" si="5"/>
+        <v>351</v>
+      </c>
+    </row>
+    <row r="353" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A353" s="4" t="s">
         <v>349</v>
-      </c>
-    </row>
-    <row r="351" spans="1:2" ht="15.6">
-      <c r="A351" s="7" t="s">
-        <v>349</v>
-      </c>
-      <c r="B351" s="3">
-        <f t="shared" si="5"/>
-        <v>350</v>
-      </c>
-    </row>
-    <row r="352" spans="1:2" ht="15.6">
-      <c r="A352" s="7" t="s">
-        <v>350</v>
-      </c>
-      <c r="B352" s="3">
-        <f t="shared" si="5"/>
-        <v>351</v>
-      </c>
-    </row>
-    <row r="353" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A353" s="7" t="s">
-        <v>351</v>
       </c>
       <c r="B353" s="3">
         <f t="shared" si="5"/>
@@ -4984,7 +4999,7 @@
     </row>
     <row r="354" spans="1:2" ht="15.6">
       <c r="A354" s="4" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B354" s="3">
         <f t="shared" si="5"/>
@@ -4993,7 +5008,7 @@
     </row>
     <row r="355" spans="1:2" ht="15.6">
       <c r="A355" s="4" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B355" s="3">
         <f t="shared" si="5"/>
@@ -5002,7 +5017,7 @@
     </row>
     <row r="356" spans="1:2" ht="15.6">
       <c r="A356" s="4" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B356" s="3">
         <f t="shared" si="5"/>
@@ -5011,7 +5026,7 @@
     </row>
     <row r="357" spans="1:2" ht="15.6">
       <c r="A357" s="4" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B357" s="3">
         <f t="shared" si="5"/>
@@ -5020,7 +5035,7 @@
     </row>
     <row r="358" spans="1:2" ht="15.6">
       <c r="A358" s="4" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B358" s="3">
         <f t="shared" si="5"/>
@@ -5029,7 +5044,7 @@
     </row>
     <row r="359" spans="1:2" ht="15.6">
       <c r="A359" s="4" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B359" s="3">
         <f t="shared" si="5"/>
@@ -5038,7 +5053,7 @@
     </row>
     <row r="360" spans="1:2" ht="15.6">
       <c r="A360" s="4" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B360" s="3">
         <f t="shared" si="5"/>
@@ -5047,7 +5062,7 @@
     </row>
     <row r="361" spans="1:2" ht="15.6">
       <c r="A361" s="4" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B361" s="3">
         <f t="shared" si="5"/>
@@ -5056,7 +5071,7 @@
     </row>
     <row r="362" spans="1:2" ht="15.6">
       <c r="A362" s="4" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B362" s="3">
         <f t="shared" si="5"/>
@@ -5065,7 +5080,7 @@
     </row>
     <row r="363" spans="1:2" ht="15.6">
       <c r="A363" s="4" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B363" s="3">
         <f t="shared" si="5"/>
@@ -5074,7 +5089,7 @@
     </row>
     <row r="364" spans="1:2" ht="15.6">
       <c r="A364" s="4" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B364" s="3">
         <f t="shared" si="5"/>
@@ -5083,7 +5098,7 @@
     </row>
     <row r="365" spans="1:2" ht="15.6">
       <c r="A365" s="4" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B365" s="3">
         <f t="shared" si="5"/>
@@ -5092,7 +5107,7 @@
     </row>
     <row r="366" spans="1:2" ht="15.6">
       <c r="A366" s="4" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B366" s="3">
         <f t="shared" si="5"/>
@@ -5101,7 +5116,7 @@
     </row>
     <row r="367" spans="1:2" ht="15.6">
       <c r="A367" s="4" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B367" s="3">
         <f t="shared" si="5"/>
@@ -5110,7 +5125,7 @@
     </row>
     <row r="368" spans="1:2" ht="15.6">
       <c r="A368" s="4" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B368" s="3">
         <f t="shared" si="5"/>
@@ -5119,7 +5134,7 @@
     </row>
     <row r="369" spans="1:2" ht="15.6">
       <c r="A369" s="4" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B369" s="3">
         <f t="shared" si="5"/>
@@ -5128,7 +5143,7 @@
     </row>
     <row r="370" spans="1:2" ht="15.6">
       <c r="A370" s="4" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B370" s="3">
         <f t="shared" si="5"/>
@@ -5137,7 +5152,7 @@
     </row>
     <row r="371" spans="1:2" ht="15.6">
       <c r="A371" s="4" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B371" s="3">
         <f t="shared" si="5"/>
@@ -5146,7 +5161,7 @@
     </row>
     <row r="372" spans="1:2" ht="15.6">
       <c r="A372" s="4" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B372" s="3">
         <f t="shared" si="5"/>
@@ -5155,7 +5170,7 @@
     </row>
     <row r="373" spans="1:2" ht="15.6">
       <c r="A373" s="4" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B373" s="3">
         <f t="shared" si="5"/>
@@ -5164,7 +5179,7 @@
     </row>
     <row r="374" spans="1:2" ht="15.6">
       <c r="A374" s="4" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B374" s="3">
         <f t="shared" si="5"/>
@@ -5173,7 +5188,7 @@
     </row>
     <row r="375" spans="1:2" ht="15.6">
       <c r="A375" s="4" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B375" s="3">
         <f t="shared" si="5"/>
@@ -5182,7 +5197,7 @@
     </row>
     <row r="376" spans="1:2" ht="15.6">
       <c r="A376" s="4" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B376" s="3">
         <f t="shared" si="5"/>
@@ -5191,7 +5206,7 @@
     </row>
     <row r="377" spans="1:2" ht="15.6">
       <c r="A377" s="4" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B377" s="3">
         <f t="shared" si="5"/>
@@ -5200,7 +5215,7 @@
     </row>
     <row r="378" spans="1:2" ht="15.6">
       <c r="A378" s="4" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B378" s="3">
         <f t="shared" si="5"/>
@@ -5209,7 +5224,7 @@
     </row>
     <row r="379" spans="1:2" ht="15.6">
       <c r="A379" s="4" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B379" s="3">
         <f t="shared" si="5"/>
@@ -5218,7 +5233,7 @@
     </row>
     <row r="380" spans="1:2" ht="15.6">
       <c r="A380" s="4" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B380" s="3">
         <f t="shared" si="5"/>
@@ -5227,7 +5242,7 @@
     </row>
     <row r="381" spans="1:2" ht="15.6">
       <c r="A381" s="4" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B381" s="3">
         <f t="shared" si="5"/>
@@ -5236,7 +5251,7 @@
     </row>
     <row r="382" spans="1:2" ht="15.6">
       <c r="A382" s="4" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B382" s="3">
         <f t="shared" si="5"/>
@@ -5245,7 +5260,7 @@
     </row>
     <row r="383" spans="1:2" ht="15.6">
       <c r="A383" s="4" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B383" s="3">
         <f t="shared" si="5"/>
@@ -5254,7 +5269,7 @@
     </row>
     <row r="384" spans="1:2" ht="15.6">
       <c r="A384" s="4" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B384" s="3">
         <f t="shared" si="5"/>
@@ -5263,7 +5278,7 @@
     </row>
     <row r="385" spans="1:2" ht="15.6">
       <c r="A385" s="4" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B385" s="3">
         <f t="shared" si="5"/>
@@ -5272,7 +5287,7 @@
     </row>
     <row r="386" spans="1:2" ht="15.6">
       <c r="A386" s="4" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B386" s="3">
         <f t="shared" si="5"/>
@@ -5281,7 +5296,7 @@
     </row>
     <row r="387" spans="1:2" ht="15.6">
       <c r="A387" s="4" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B387" s="3">
         <f t="shared" si="5"/>
@@ -5290,16 +5305,16 @@
     </row>
     <row r="388" spans="1:2" ht="15.6">
       <c r="A388" s="4" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B388" s="3">
-        <f t="shared" ref="B388:B436" si="6">B387+1</f>
+        <f t="shared" ref="B388:B444" si="6">B387+1</f>
         <v>387</v>
       </c>
     </row>
     <row r="389" spans="1:2" ht="15.6">
       <c r="A389" s="4" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="B389" s="3">
         <f t="shared" si="6"/>
@@ -5308,7 +5323,7 @@
     </row>
     <row r="390" spans="1:2" ht="15.6">
       <c r="A390" s="4" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B390" s="3">
         <f t="shared" si="6"/>
@@ -5317,7 +5332,7 @@
     </row>
     <row r="391" spans="1:2" ht="15.6">
       <c r="A391" s="4" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B391" s="3">
         <f t="shared" si="6"/>
@@ -5325,8 +5340,8 @@
       </c>
     </row>
     <row r="392" spans="1:2" ht="15.6">
-      <c r="A392" s="4" t="s">
-        <v>390</v>
+      <c r="A392" s="5" t="s">
+        <v>388</v>
       </c>
       <c r="B392" s="3">
         <f t="shared" si="6"/>
@@ -5334,8 +5349,8 @@
       </c>
     </row>
     <row r="393" spans="1:2" ht="15.6">
-      <c r="A393" s="4" t="s">
-        <v>391</v>
+      <c r="A393" s="5" t="s">
+        <v>389</v>
       </c>
       <c r="B393" s="3">
         <f t="shared" si="6"/>
@@ -5343,8 +5358,8 @@
       </c>
     </row>
     <row r="394" spans="1:2" ht="15.6">
-      <c r="A394" s="4" t="s">
-        <v>392</v>
+      <c r="A394" s="5" t="s">
+        <v>390</v>
       </c>
       <c r="B394" s="3">
         <f t="shared" si="6"/>
@@ -5352,8 +5367,8 @@
       </c>
     </row>
     <row r="395" spans="1:2" ht="15.6">
-      <c r="A395" s="4" t="s">
-        <v>393</v>
+      <c r="A395" s="7" t="s">
+        <v>391</v>
       </c>
       <c r="B395" s="3">
         <f t="shared" si="6"/>
@@ -5361,8 +5376,8 @@
       </c>
     </row>
     <row r="396" spans="1:2" ht="15.6">
-      <c r="A396" s="4" t="s">
-        <v>394</v>
+      <c r="A396" s="7" t="s">
+        <v>392</v>
       </c>
       <c r="B396" s="3">
         <f t="shared" si="6"/>
@@ -5371,7 +5386,7 @@
     </row>
     <row r="397" spans="1:2" ht="15.6">
       <c r="A397" s="5" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B397" s="3">
         <f t="shared" si="6"/>
@@ -5380,7 +5395,7 @@
     </row>
     <row r="398" spans="1:2" ht="15.6">
       <c r="A398" s="5" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B398" s="3">
         <f t="shared" si="6"/>
@@ -5389,7 +5404,7 @@
     </row>
     <row r="399" spans="1:2" ht="15.6">
       <c r="A399" s="5" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="B399" s="3">
         <f t="shared" si="6"/>
@@ -5397,8 +5412,8 @@
       </c>
     </row>
     <row r="400" spans="1:2" ht="15.6">
-      <c r="A400" s="7" t="s">
-        <v>398</v>
+      <c r="A400" s="5" t="s">
+        <v>396</v>
       </c>
       <c r="B400" s="3">
         <f t="shared" si="6"/>
@@ -5406,8 +5421,8 @@
       </c>
     </row>
     <row r="401" spans="1:2" ht="15.6">
-      <c r="A401" s="7" t="s">
-        <v>399</v>
+      <c r="A401" s="5" t="s">
+        <v>397</v>
       </c>
       <c r="B401" s="3">
         <f t="shared" si="6"/>
@@ -5416,7 +5431,7 @@
     </row>
     <row r="402" spans="1:2" ht="15.6">
       <c r="A402" s="5" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="B402" s="3">
         <f t="shared" si="6"/>
@@ -5425,7 +5440,7 @@
     </row>
     <row r="403" spans="1:2" ht="15.6">
       <c r="A403" s="5" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B403" s="3">
         <f t="shared" si="6"/>
@@ -5434,7 +5449,7 @@
     </row>
     <row r="404" spans="1:2" ht="15.6">
       <c r="A404" s="5" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B404" s="3">
         <f t="shared" si="6"/>
@@ -5443,7 +5458,7 @@
     </row>
     <row r="405" spans="1:2" ht="15.6">
       <c r="A405" s="5" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B405" s="3">
         <f t="shared" si="6"/>
@@ -5452,7 +5467,7 @@
     </row>
     <row r="406" spans="1:2" ht="15.6">
       <c r="A406" s="5" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B406" s="3">
         <f t="shared" si="6"/>
@@ -5461,7 +5476,7 @@
     </row>
     <row r="407" spans="1:2" ht="15.6">
       <c r="A407" s="5" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="B407" s="3">
         <f t="shared" si="6"/>
@@ -5470,7 +5485,7 @@
     </row>
     <row r="408" spans="1:2" ht="15.6">
       <c r="A408" s="5" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B408" s="3">
         <f t="shared" si="6"/>
@@ -5479,7 +5494,7 @@
     </row>
     <row r="409" spans="1:2" ht="15.6">
       <c r="A409" s="5" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B409" s="3">
         <f t="shared" si="6"/>
@@ -5488,7 +5503,7 @@
     </row>
     <row r="410" spans="1:2" ht="16.5" customHeight="1">
       <c r="A410" s="5" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B410" s="3">
         <f t="shared" si="6"/>
@@ -5497,7 +5512,7 @@
     </row>
     <row r="411" spans="1:2" ht="16.5" customHeight="1">
       <c r="A411" s="5" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="B411" s="3">
         <f t="shared" si="6"/>
@@ -5506,7 +5521,7 @@
     </row>
     <row r="412" spans="1:2" ht="16.5" customHeight="1">
       <c r="A412" s="5" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B412" s="3">
         <f t="shared" si="6"/>
@@ -5515,7 +5530,7 @@
     </row>
     <row r="413" spans="1:2" ht="16.5" customHeight="1">
       <c r="A413" s="5" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="B413" s="3">
         <f t="shared" si="6"/>
@@ -5524,7 +5539,7 @@
     </row>
     <row r="414" spans="1:2" ht="16.5" customHeight="1">
       <c r="A414" s="5" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B414" s="3">
         <f t="shared" si="6"/>
@@ -5533,7 +5548,7 @@
     </row>
     <row r="415" spans="1:2" ht="16.5" customHeight="1">
       <c r="A415" s="5" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B415" s="3">
         <f t="shared" si="6"/>
@@ -5542,7 +5557,7 @@
     </row>
     <row r="416" spans="1:2" ht="16.5" customHeight="1">
       <c r="A416" s="5" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B416" s="3">
         <f t="shared" si="6"/>
@@ -5550,8 +5565,8 @@
       </c>
     </row>
     <row r="417" spans="1:2" ht="16.5" customHeight="1">
-      <c r="A417" s="5" t="s">
-        <v>415</v>
+      <c r="A417" s="4" t="s">
+        <v>413</v>
       </c>
       <c r="B417" s="3">
         <f t="shared" si="6"/>
@@ -5559,8 +5574,8 @@
       </c>
     </row>
     <row r="418" spans="1:2" ht="16.5" customHeight="1">
-      <c r="A418" s="5" t="s">
-        <v>416</v>
+      <c r="A418" s="4" t="s">
+        <v>414</v>
       </c>
       <c r="B418" s="3">
         <f t="shared" si="6"/>
@@ -5568,8 +5583,8 @@
       </c>
     </row>
     <row r="419" spans="1:2" ht="16.5" customHeight="1">
-      <c r="A419" s="5" t="s">
-        <v>417</v>
+      <c r="A419" s="4" t="s">
+        <v>415</v>
       </c>
       <c r="B419" s="3">
         <f t="shared" si="6"/>
@@ -5577,8 +5592,8 @@
       </c>
     </row>
     <row r="420" spans="1:2" ht="16.5" customHeight="1">
-      <c r="A420" s="5" t="s">
-        <v>418</v>
+      <c r="A420" s="4" t="s">
+        <v>416</v>
       </c>
       <c r="B420" s="3">
         <f t="shared" si="6"/>
@@ -5586,8 +5601,8 @@
       </c>
     </row>
     <row r="421" spans="1:2" ht="16.5" customHeight="1">
-      <c r="A421" s="5" t="s">
-        <v>419</v>
+      <c r="A421" s="4" t="s">
+        <v>417</v>
       </c>
       <c r="B421" s="3">
         <f t="shared" si="6"/>
@@ -5596,7 +5611,7 @@
     </row>
     <row r="422" spans="1:2" ht="16.5" customHeight="1">
       <c r="A422" s="4" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B422" s="3">
         <f t="shared" si="6"/>
@@ -5605,7 +5620,7 @@
     </row>
     <row r="423" spans="1:2" ht="16.5" customHeight="1">
       <c r="A423" s="4" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="B423" s="3">
         <f t="shared" si="6"/>
@@ -5614,7 +5629,7 @@
     </row>
     <row r="424" spans="1:2" ht="16.5" customHeight="1">
       <c r="A424" s="4" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B424" s="3">
         <f t="shared" si="6"/>
@@ -5623,7 +5638,7 @@
     </row>
     <row r="425" spans="1:2" ht="16.5" customHeight="1">
       <c r="A425" s="4" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="B425" s="3">
         <f t="shared" si="6"/>
@@ -5632,7 +5647,7 @@
     </row>
     <row r="426" spans="1:2" ht="16.5" customHeight="1">
       <c r="A426" s="4" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B426" s="3">
         <f t="shared" si="6"/>
@@ -5641,7 +5656,7 @@
     </row>
     <row r="427" spans="1:2" ht="16.5" customHeight="1">
       <c r="A427" s="4" t="s">
-        <v>425</v>
+        <v>400</v>
       </c>
       <c r="B427" s="3">
         <f t="shared" si="6"/>
@@ -5650,7 +5665,7 @@
     </row>
     <row r="428" spans="1:2" ht="16.5" customHeight="1">
       <c r="A428" s="4" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="B428" s="3">
         <f t="shared" si="6"/>
@@ -5659,7 +5674,7 @@
     </row>
     <row r="429" spans="1:2" ht="16.5" customHeight="1">
       <c r="A429" s="4" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="B429" s="3">
         <f t="shared" si="6"/>
@@ -5668,7 +5683,7 @@
     </row>
     <row r="430" spans="1:2" ht="16.5" customHeight="1">
       <c r="A430" s="4" t="s">
-        <v>428</v>
+        <v>409</v>
       </c>
       <c r="B430" s="3">
         <f t="shared" si="6"/>
@@ -5677,7 +5692,7 @@
     </row>
     <row r="431" spans="1:2" ht="16.5" customHeight="1">
       <c r="A431" s="4" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="B431" s="3">
         <f t="shared" si="6"/>
@@ -5686,7 +5701,7 @@
     </row>
     <row r="432" spans="1:2" ht="16.5" customHeight="1">
       <c r="A432" s="4" t="s">
-        <v>407</v>
+        <v>430</v>
       </c>
       <c r="B432" s="3">
         <f t="shared" si="6"/>
@@ -5695,7 +5710,7 @@
     </row>
     <row r="433" spans="1:2" ht="16.5" customHeight="1">
       <c r="A433" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B433" s="3">
         <f t="shared" si="6"/>
@@ -5704,7 +5719,7 @@
     </row>
     <row r="434" spans="1:2" ht="16.5" customHeight="1">
       <c r="A434" s="4" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B434" s="3">
         <f t="shared" si="6"/>
@@ -5713,7 +5728,7 @@
     </row>
     <row r="435" spans="1:2" ht="16.5" customHeight="1">
       <c r="A435" s="4" t="s">
-        <v>416</v>
+        <v>433</v>
       </c>
       <c r="B435" s="3">
         <f t="shared" si="6"/>
@@ -5722,11 +5737,83 @@
     </row>
     <row r="436" spans="1:2" ht="16.5" customHeight="1">
       <c r="A436" s="4" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B436" s="3">
         <f t="shared" si="6"/>
         <v>435</v>
+      </c>
+    </row>
+    <row r="437" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A437" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="B437" s="3">
+        <f t="shared" si="6"/>
+        <v>436</v>
+      </c>
+    </row>
+    <row r="438" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A438" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="B438" s="3">
+        <f t="shared" si="6"/>
+        <v>437</v>
+      </c>
+    </row>
+    <row r="439" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A439" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="B439" s="3">
+        <f t="shared" si="6"/>
+        <v>438</v>
+      </c>
+    </row>
+    <row r="440" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A440" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="B440" s="3">
+        <f t="shared" si="6"/>
+        <v>439</v>
+      </c>
+    </row>
+    <row r="441" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A441" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="B441" s="3">
+        <f t="shared" si="6"/>
+        <v>440</v>
+      </c>
+    </row>
+    <row r="442" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A442" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="B442" s="3">
+        <f t="shared" si="6"/>
+        <v>441</v>
+      </c>
+    </row>
+    <row r="443" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A443" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="B443" s="3">
+        <f t="shared" si="6"/>
+        <v>442</v>
+      </c>
+    </row>
+    <row r="444" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A444" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="B444" s="3">
+        <f t="shared" si="6"/>
+        <v>443</v>
       </c>
     </row>
   </sheetData>

</xml_diff>